<commit_message>
Agregar costos y margen a catalogo
</commit_message>
<xml_diff>
--- a/data/catalogo_productos.xlsx
+++ b/data/catalogo_productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eaton-my.sharepoint.com/personal/arelycastillo_eaton_com/Documents/Documents/GitHub/Eaton/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="221" documentId="8_{FA424185-D530-44FF-BEF1-1D3F8B302D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{33750515-3870-4167-971B-F7306F2CBFE4}"/>
+  <xr:revisionPtr revIDLastSave="222" documentId="8_{FA424185-D530-44FF-BEF1-1D3F8B302D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C53D82F-0031-4DDF-AF9D-39F9D4B0D0C0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{E356A83D-CAB3-4D69-8690-2DF2AB7B7938}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="11" activeTab="18" xr2:uid="{E356A83D-CAB3-4D69-8690-2DF2AB7B7938}"/>
   </bookViews>
   <sheets>
     <sheet name="Estructura" sheetId="9" r:id="rId1"/>
@@ -11631,7 +11631,6 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C72381-812D-42EC-84BC-3CAA921F011E}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G93"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -11664,7 +11663,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>425</v>
       </c>
@@ -11687,7 +11686,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>427</v>
       </c>
@@ -11710,7 +11709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>429</v>
       </c>
@@ -11733,7 +11732,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>430</v>
       </c>
@@ -11756,7 +11755,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>431</v>
       </c>
@@ -11779,7 +11778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>432</v>
       </c>
@@ -11802,7 +11801,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>433</v>
       </c>
@@ -11825,7 +11824,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>434</v>
       </c>
@@ -11848,7 +11847,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>435</v>
       </c>
@@ -11871,7 +11870,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>436</v>
       </c>
@@ -11894,7 +11893,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>445</v>
       </c>
@@ -11917,7 +11916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>446</v>
       </c>
@@ -11940,7 +11939,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>447</v>
       </c>
@@ -11963,7 +11962,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>448</v>
       </c>
@@ -11986,7 +11985,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>449</v>
       </c>
@@ -12354,7 +12353,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>485</v>
       </c>
@@ -12377,7 +12376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>487</v>
       </c>
@@ -12400,7 +12399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>488</v>
       </c>
@@ -12423,7 +12422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>491</v>
       </c>
@@ -12446,7 +12445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>493</v>
       </c>
@@ -12469,7 +12468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>494</v>
       </c>
@@ -12492,7 +12491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>495</v>
       </c>
@@ -12515,7 +12514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>496</v>
       </c>
@@ -12538,7 +12537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>497</v>
       </c>
@@ -12561,7 +12560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>498</v>
       </c>
@@ -12584,7 +12583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>499</v>
       </c>
@@ -12607,7 +12606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>507</v>
       </c>
@@ -12630,7 +12629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>509</v>
       </c>
@@ -12653,7 +12652,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>511</v>
       </c>
@@ -12676,7 +12675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>513</v>
       </c>
@@ -12699,7 +12698,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>515</v>
       </c>
@@ -12722,7 +12721,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>516</v>
       </c>
@@ -12745,7 +12744,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>517</v>
       </c>
@@ -12768,7 +12767,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>518</v>
       </c>
@@ -12791,7 +12790,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>519</v>
       </c>
@@ -12814,7 +12813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>525</v>
       </c>
@@ -12837,7 +12836,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>526</v>
       </c>
@@ -12860,7 +12859,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>529</v>
       </c>
@@ -12883,7 +12882,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>531</v>
       </c>
@@ -12906,7 +12905,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>532</v>
       </c>
@@ -12929,7 +12928,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>533</v>
       </c>
@@ -13297,7 +13296,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>563</v>
       </c>
@@ -13320,7 +13319,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>564</v>
       </c>
@@ -13343,7 +13342,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>565</v>
       </c>
@@ -13366,7 +13365,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>566</v>
       </c>
@@ -13389,7 +13388,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>567</v>
       </c>
@@ -13412,7 +13411,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>573</v>
       </c>
@@ -13435,7 +13434,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>575</v>
       </c>
@@ -13458,7 +13457,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>576</v>
       </c>
@@ -13481,7 +13480,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>577</v>
       </c>
@@ -13781,13 +13780,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G93" xr:uid="{F7C72381-812D-42EC-84BC-3CAA921F011E}">
-    <filterColumn colId="6">
-      <filters>
-        <filter val="3"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G93" xr:uid="{F7C72381-812D-42EC-84BC-3CAA921F011E}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Costos y Margen IZMX
</commit_message>
<xml_diff>
--- a/data/catalogo_productos.xlsx
+++ b/data/catalogo_productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eaton-my.sharepoint.com/personal/arelycastillo_eaton_com/Documents/Documents/GitHub/Eaton/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="222" documentId="8_{FA424185-D530-44FF-BEF1-1D3F8B302D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C53D82F-0031-4DDF-AF9D-39F9D4B0D0C0}"/>
+  <xr:revisionPtr revIDLastSave="250" documentId="8_{FA424185-D530-44FF-BEF1-1D3F8B302D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE11FF66-5101-4E97-ABF3-21CB180E892A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="11" activeTab="18" xr2:uid="{E356A83D-CAB3-4D69-8690-2DF2AB7B7938}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="4" xr2:uid="{E356A83D-CAB3-4D69-8690-2DF2AB7B7938}"/>
   </bookViews>
   <sheets>
     <sheet name="Estructura" sheetId="9" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2100" uniqueCount="765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="765">
   <si>
     <t>Catalogo</t>
   </si>
@@ -2461,7 +2461,7 @@
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2502,6 +2502,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -2520,6 +2526,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16538,16 +16548,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33FF069F-11F0-41FB-B939-51B5F45B8CB2}">
-  <dimension ref="A1:E111"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13" style="17" customWidth="1"/>
+    <col min="6" max="6" width="12.54296875" style="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -16560,11 +16572,17 @@
       <c r="D1" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="26" t="s">
+        <v>747</v>
+      </c>
+      <c r="F1" s="13" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G1" s="24" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>689</v>
       </c>
@@ -16577,11 +16595,19 @@
       <c r="D2" s="11" t="s">
         <v>695</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="27">
+        <f>1605.72*18</f>
+        <v>28902.959999999999</v>
+      </c>
+      <c r="F2" s="12">
         <v>103121</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G2" s="19">
+        <f>ROUND(((F2-E2)/F2),4)</f>
+        <v>0.71970000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>690</v>
       </c>
@@ -16594,11 +16620,19 @@
       <c r="D3" s="11" t="s">
         <v>695</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="27">
+        <f>2372.73*18</f>
+        <v>42709.14</v>
+      </c>
+      <c r="F3" s="12">
         <v>118541</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G3" s="19">
+        <f t="shared" ref="G3:G14" si="0">ROUND(((F3-E3)/F3),4)</f>
+        <v>0.63970000000000005</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="11" t="s">
         <v>691</v>
       </c>
@@ -16611,11 +16645,19 @@
       <c r="D4" s="11" t="s">
         <v>695</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="27">
+        <f>2482.17*18</f>
+        <v>44679.06</v>
+      </c>
+      <c r="F4" s="12">
         <v>135356</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G4" s="19">
+        <f t="shared" si="0"/>
+        <v>0.66990000000000005</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>692</v>
       </c>
@@ -16628,11 +16670,19 @@
       <c r="D5" s="11" t="s">
         <v>695</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="27">
+        <f>2081.55*18</f>
+        <v>37467.9</v>
+      </c>
+      <c r="F5" s="12">
         <v>128574</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G5" s="19">
+        <f t="shared" si="0"/>
+        <v>0.70860000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>693</v>
       </c>
@@ -16645,11 +16695,19 @@
       <c r="D6" s="11" t="s">
         <v>695</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="27">
+        <f>3365*18</f>
+        <v>60570</v>
+      </c>
+      <c r="F6" s="12">
         <v>145962</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G6" s="19">
+        <f t="shared" si="0"/>
+        <v>0.58499999999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>694</v>
       </c>
@@ -16662,11 +16720,19 @@
       <c r="D7" s="11" t="s">
         <v>695</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="27">
+        <f>3762.16*18</f>
+        <v>67718.880000000005</v>
+      </c>
+      <c r="F7" s="12">
         <v>163173</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G7" s="19">
+        <f t="shared" si="0"/>
+        <v>0.58499999999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>696</v>
       </c>
@@ -16679,11 +16745,19 @@
       <c r="D8" s="11" t="s">
         <v>704</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="27">
+        <f>1749.21*18</f>
+        <v>31485.78</v>
+      </c>
+      <c r="F8" s="12">
         <v>115840</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G8" s="19">
+        <f t="shared" si="0"/>
+        <v>0.72819999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>697</v>
       </c>
@@ -16696,11 +16770,19 @@
       <c r="D9" s="11" t="s">
         <v>704</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="27">
+        <f>2535.37*18</f>
+        <v>45636.659999999996</v>
+      </c>
+      <c r="F9" s="12">
         <v>131702</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G9" s="19">
+        <f t="shared" si="0"/>
+        <v>0.65349999999999997</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>698</v>
       </c>
@@ -16713,11 +16795,19 @@
       <c r="D10" s="11" t="s">
         <v>704</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="27">
+        <f>2644.81*18</f>
+        <v>47606.58</v>
+      </c>
+      <c r="F10" s="12">
         <v>148391</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G10" s="19">
+        <f t="shared" si="0"/>
+        <v>0.67920000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>699</v>
       </c>
@@ -16730,11 +16820,19 @@
       <c r="D11" s="11" t="s">
         <v>704</v>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="27">
+        <f>2225.04*18</f>
+        <v>40050.720000000001</v>
+      </c>
+      <c r="F11" s="12">
         <v>141557</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G11" s="19">
+        <f t="shared" si="0"/>
+        <v>0.71709999999999996</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>700</v>
       </c>
@@ -16747,11 +16845,19 @@
       <c r="D12" s="11" t="s">
         <v>704</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="27">
+        <f>3527.64*18</f>
+        <v>63497.52</v>
+      </c>
+      <c r="F12" s="12">
         <v>159273</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G12" s="19">
+        <f t="shared" si="0"/>
+        <v>0.60129999999999995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>701</v>
       </c>
@@ -16764,11 +16870,19 @@
       <c r="D13" s="11" t="s">
         <v>704</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="27">
+        <f>3924.8*18</f>
+        <v>70646.400000000009</v>
+      </c>
+      <c r="F13" s="12">
         <v>178319</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G13" s="19">
+        <f t="shared" si="0"/>
+        <v>0.6038</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>702</v>
       </c>
@@ -16781,591 +16895,696 @@
       <c r="D14" t="s">
         <v>703</v>
       </c>
-      <c r="E14" s="12">
+      <c r="E14" s="17">
+        <f>309.63*18</f>
+        <v>5573.34</v>
+      </c>
+      <c r="F14" s="12">
         <v>7067</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G14" s="19">
+        <f t="shared" si="0"/>
+        <v>0.2114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E15" s="27"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E16" s="27"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E17" s="27"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="11"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E18" s="27"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="11"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E19" s="27"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="11"/>
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E20" s="27"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="11"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E21" s="27"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="11"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E22" s="27"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="11"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E23" s="27"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="11"/>
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E24" s="27"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="11"/>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E25" s="27"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="11"/>
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E26" s="27"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="11"/>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E27" s="27"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="11"/>
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E28" s="27"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="11"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E29" s="27"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="11"/>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E30" s="27"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="11"/>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E31" s="27"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="11"/>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E32" s="27"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="11"/>
       <c r="B33" s="11"/>
       <c r="C33" s="11"/>
       <c r="D33" s="11"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E33" s="27"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="11"/>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E34" s="27"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="11"/>
       <c r="B35" s="11"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E35" s="27"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="11"/>
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E36" s="27"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="11"/>
       <c r="B37" s="11"/>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E37" s="27"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="11"/>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E38" s="27"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="11"/>
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E39" s="27"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="11"/>
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E40" s="27"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="11"/>
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E41" s="27"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="11"/>
       <c r="B42" s="11"/>
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E42" s="27"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="11"/>
       <c r="B43" s="11"/>
       <c r="C43" s="11"/>
       <c r="D43" s="11"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E43" s="27"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="11"/>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
       <c r="D44" s="11"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E44" s="27"/>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="11"/>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E45" s="27"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="11"/>
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
       <c r="D46" s="11"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E46" s="27"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="11"/>
       <c r="B47" s="11"/>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E47" s="27"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
       <c r="D48" s="11"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E48" s="27"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="11"/>
       <c r="B49" s="11"/>
       <c r="C49" s="11"/>
       <c r="D49" s="11"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E49" s="27"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="11"/>
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
       <c r="D50" s="11"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E50" s="27"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="11"/>
       <c r="B51" s="11"/>
       <c r="C51" s="11"/>
       <c r="D51" s="11"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E51" s="27"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="11"/>
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
       <c r="D52" s="11"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E52" s="27"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="11"/>
       <c r="B53" s="11"/>
       <c r="C53" s="11"/>
       <c r="D53" s="11"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E53" s="27"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="11"/>
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E54" s="27"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="11"/>
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
       <c r="D55" s="11"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E55" s="27"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="11"/>
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E56" s="27"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="11"/>
       <c r="B57" s="11"/>
       <c r="C57" s="11"/>
       <c r="D57" s="11"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E57" s="27"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="11"/>
       <c r="B58" s="11"/>
       <c r="C58" s="11"/>
       <c r="D58" s="11"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E58" s="27"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="11"/>
       <c r="B59" s="11"/>
       <c r="C59" s="11"/>
       <c r="D59" s="11"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E59" s="27"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="11"/>
       <c r="B60" s="11"/>
       <c r="C60" s="11"/>
       <c r="D60" s="11"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E60" s="27"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="11"/>
       <c r="B61" s="11"/>
       <c r="C61" s="11"/>
       <c r="D61" s="11"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E61" s="27"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="11"/>
       <c r="B62" s="11"/>
       <c r="C62" s="11"/>
       <c r="D62" s="11"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E62" s="27"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="11"/>
       <c r="B63" s="11"/>
       <c r="C63" s="11"/>
       <c r="D63" s="11"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E63" s="27"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="11"/>
       <c r="B64" s="11"/>
       <c r="C64" s="11"/>
       <c r="D64" s="11"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E64" s="27"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="11"/>
       <c r="B65" s="11"/>
       <c r="C65" s="11"/>
       <c r="D65" s="11"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E65" s="27"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="11"/>
       <c r="B66" s="11"/>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E66" s="27"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="11"/>
       <c r="B67" s="11"/>
       <c r="C67" s="11"/>
       <c r="D67" s="11"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E67" s="27"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="11"/>
       <c r="B68" s="11"/>
       <c r="C68" s="11"/>
       <c r="D68" s="11"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E68" s="27"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="11"/>
       <c r="B69" s="11"/>
       <c r="C69" s="11"/>
       <c r="D69" s="11"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E69" s="27"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="11"/>
       <c r="B70" s="11"/>
       <c r="C70" s="11"/>
       <c r="D70" s="11"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E70" s="27"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="11"/>
       <c r="B71" s="11"/>
       <c r="C71" s="11"/>
       <c r="D71" s="11"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E71" s="27"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="11"/>
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
       <c r="D72" s="11"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E72" s="27"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="11"/>
       <c r="B73" s="11"/>
       <c r="C73" s="11"/>
       <c r="D73" s="11"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E73" s="27"/>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="11"/>
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
       <c r="D74" s="11"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E74" s="27"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="11"/>
       <c r="B75" s="11"/>
       <c r="C75" s="11"/>
       <c r="D75" s="11"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E75" s="27"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="11"/>
       <c r="B76" s="11"/>
       <c r="C76" s="11"/>
       <c r="D76" s="11"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E76" s="27"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="11"/>
       <c r="B77" s="11"/>
       <c r="C77" s="11"/>
       <c r="D77" s="11"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E77" s="27"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="11"/>
       <c r="B78" s="11"/>
       <c r="C78" s="11"/>
       <c r="D78" s="11"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E78" s="27"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="11"/>
       <c r="B79" s="11"/>
       <c r="C79" s="11"/>
       <c r="D79" s="11"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E79" s="27"/>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="11"/>
       <c r="B80" s="11"/>
       <c r="C80" s="11"/>
       <c r="D80" s="11"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E80" s="27"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="11"/>
       <c r="B81" s="11"/>
       <c r="C81" s="11"/>
       <c r="D81" s="11"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E81" s="27"/>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="11"/>
       <c r="B82" s="11"/>
       <c r="C82" s="11"/>
       <c r="D82" s="11"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E82" s="27"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="11"/>
       <c r="B83" s="11"/>
       <c r="C83" s="11"/>
       <c r="D83" s="11"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E83" s="27"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="11"/>
       <c r="B84" s="11"/>
       <c r="C84" s="11"/>
       <c r="D84" s="11"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E84" s="27"/>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="11"/>
       <c r="B85" s="11"/>
       <c r="C85" s="11"/>
       <c r="D85" s="11"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E85" s="27"/>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="11"/>
       <c r="B86" s="11"/>
       <c r="C86" s="11"/>
       <c r="D86" s="11"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E86" s="27"/>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="11"/>
       <c r="B87" s="11"/>
       <c r="C87" s="11"/>
       <c r="D87" s="11"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E87" s="27"/>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="11"/>
       <c r="B88" s="11"/>
       <c r="C88" s="11"/>
       <c r="D88" s="11"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E88" s="27"/>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="11"/>
       <c r="B89" s="11"/>
       <c r="C89" s="11"/>
       <c r="D89" s="11"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E89" s="27"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="11"/>
       <c r="B90" s="11"/>
       <c r="C90" s="11"/>
       <c r="D90" s="11"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E90" s="27"/>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="11"/>
       <c r="B91" s="11"/>
       <c r="C91" s="11"/>
       <c r="D91" s="11"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E91" s="27"/>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="11"/>
       <c r="B92" s="11"/>
       <c r="C92" s="11"/>
       <c r="D92" s="11"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E92" s="27"/>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="11"/>
       <c r="B93" s="11"/>
       <c r="C93" s="11"/>
       <c r="D93" s="11"/>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E93" s="27"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="11"/>
       <c r="B94" s="11"/>
       <c r="C94" s="11"/>
       <c r="D94" s="11"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E94" s="27"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="11"/>
       <c r="B95" s="11"/>
       <c r="C95" s="11"/>
       <c r="D95" s="11"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E95" s="27"/>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="11"/>
       <c r="B96" s="11"/>
       <c r="C96" s="11"/>
       <c r="D96" s="11"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E96" s="27"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="11"/>
       <c r="B97" s="11"/>
       <c r="C97" s="11"/>
       <c r="D97" s="11"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E97" s="27"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="11"/>
       <c r="B98" s="11"/>
       <c r="C98" s="11"/>
       <c r="D98" s="11"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E98" s="27"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="11"/>
       <c r="B99" s="11"/>
       <c r="C99" s="11"/>
       <c r="D99" s="11"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E99" s="27"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="11"/>
       <c r="B100" s="11"/>
       <c r="C100" s="11"/>
       <c r="D100" s="11"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E100" s="27"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="11"/>
       <c r="B101" s="11"/>
       <c r="C101" s="11"/>
       <c r="D101" s="11"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E101" s="27"/>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="11"/>
       <c r="B102" s="11"/>
       <c r="C102" s="11"/>
       <c r="D102" s="11"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E102" s="27"/>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="11"/>
       <c r="B103" s="11"/>
       <c r="C103" s="11"/>
       <c r="D103" s="11"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E103" s="27"/>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="11"/>
       <c r="B104" s="11"/>
       <c r="C104" s="11"/>
       <c r="D104" s="11"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E104" s="27"/>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="11"/>
       <c r="B105" s="11"/>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E105" s="27"/>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="11"/>
       <c r="B106" s="11"/>
       <c r="C106" s="11"/>
       <c r="D106" s="11"/>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E106" s="27"/>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="11"/>
       <c r="B107" s="11"/>
       <c r="C107" s="11"/>
       <c r="D107" s="11"/>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E107" s="27"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="11"/>
       <c r="B108" s="11"/>
       <c r="C108" s="11"/>
       <c r="D108" s="11"/>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E108" s="27"/>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="11"/>
       <c r="B109" s="11"/>
       <c r="C109" s="11"/>
       <c r="D109" s="11"/>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E109" s="27"/>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="11"/>
       <c r="B110" s="11"/>
       <c r="C110" s="11"/>
       <c r="D110" s="11"/>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E110" s="27"/>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="11"/>
       <c r="B111" s="11"/>
       <c r="C111" s="11"/>
       <c r="D111" s="11"/>
+      <c r="E111" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>